<commit_message>
feat: update city center output Excel file with new data
</commit_message>
<xml_diff>
--- a/city_center_output.xlsx
+++ b/city_center_output.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\haoning\Documents\GitHub\@buildingdata\city-center\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C5B59C2-380C-4EC6-91B4-BFF04C12E8B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2A2E2C2-3D86-4A73-8980-63A7D5697B6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1690,7 +1690,7 @@
   <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="8.59765625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="12.59765625" style="3" customWidth="1"/>
     <col min="2" max="3" width="16.59765625" style="3" customWidth="1"/>
     <col min="4" max="4" width="24.59765625" style="3" customWidth="1"/>
     <col min="5" max="5" width="8.59765625" style="3" customWidth="1"/>
@@ -2261,7 +2261,7 @@
   <dimension ref="A1:E365"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="8.59765625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="12.59765625" style="3" customWidth="1"/>
     <col min="2" max="3" width="16.59765625" style="3" customWidth="1"/>
     <col min="4" max="4" width="24.59765625" style="3" customWidth="1"/>
     <col min="5" max="5" width="8.59765625" style="3" customWidth="1"/>

</xml_diff>